<commit_message>
Refresh Auditor General and TSB Info Source data
</commit_message>
<xml_diff>
--- a/institution_registry.xlsx
+++ b/institution_registry.xlsx
@@ -21227,15 +21227,51 @@
       <c r="BH55" t="inlineStr"/>
       <c r="BI55" t="inlineStr"/>
       <c r="BJ55" t="inlineStr"/>
-      <c r="BK55" t="inlineStr"/>
-      <c r="BL55" t="inlineStr"/>
-      <c r="BM55" t="inlineStr"/>
-      <c r="BN55" t="inlineStr"/>
-      <c r="BO55" t="inlineStr"/>
-      <c r="BP55" t="inlineStr"/>
-      <c r="BQ55" t="inlineStr"/>
-      <c r="BR55" t="inlineStr"/>
-      <c r="BS55" t="inlineStr"/>
+      <c r="BK55" t="inlineStr">
+        <is>
+          <t>https://www.tsb.gc.ca/eng/divulgation-disclosure/infosource/index.html</t>
+        </is>
+      </c>
+      <c r="BL55" t="inlineStr">
+        <is>
+          <t>https://www.tsb.gc.ca/fra/divulgation-disclosure/infosource/index.html</t>
+        </is>
+      </c>
+      <c r="BM55" t="inlineStr">
+        <is>
+          <t>https://www.tsb.gc.ca/eng/divulgation-disclosure/infosource/index.html</t>
+        </is>
+      </c>
+      <c r="BN55" t="inlineStr">
+        <is>
+          <t>https://www.tsb.gc.ca/fra/divulgation-disclosure/infosource/index.html</t>
+        </is>
+      </c>
+      <c r="BO55" t="inlineStr">
+        <is>
+          <t>https://www.tsb.gc.ca/eng/divulgation-disclosure/infosource/index.html</t>
+        </is>
+      </c>
+      <c r="BP55" t="inlineStr">
+        <is>
+          <t>https://www.tsb.gc.ca/fra/divulgation-disclosure/infosource/index.html</t>
+        </is>
+      </c>
+      <c r="BQ55" t="inlineStr">
+        <is>
+          <t>https://www.tsb.gc.ca/eng/divulgation-disclosure/infosource/index.html</t>
+        </is>
+      </c>
+      <c r="BR55" t="inlineStr">
+        <is>
+          <t>https://www.tsb.gc.ca/fra/divulgation-disclosure/infosource/index.html</t>
+        </is>
+      </c>
+      <c r="BS55" t="inlineStr">
+        <is>
+          <t>Current bilingual institution pages replace legacy .asp routes that redirect to a generic splash page.</t>
+        </is>
+      </c>
       <c r="BT55" t="inlineStr">
         <is>
           <t>12-31</t>
@@ -21248,32 +21284,32 @@
       </c>
       <c r="BV55" t="inlineStr">
         <is>
-          <t>http://tsb-bst.gc.ca/eng/divulgation-disclosure/infosource/index.asp</t>
+          <t>https://www.tsb.gc.ca/eng/divulgation-disclosure/infosource/index.html</t>
         </is>
       </c>
       <c r="BW55" t="inlineStr">
         <is>
-          <t>http://tsb-bst.gc.ca/fra/divulgation-disclosure/infosource/index.asp</t>
+          <t>https://www.tsb.gc.ca/fra/divulgation-disclosure/infosource/index.html</t>
         </is>
       </c>
       <c r="BX55" t="inlineStr">
         <is>
-          <t>http://tsb-bst.gc.ca/eng/divulgation-disclosure/infosource/index.asp</t>
+          <t>https://www.tsb.gc.ca/eng/divulgation-disclosure/infosource/index.html</t>
         </is>
       </c>
       <c r="BY55" t="inlineStr">
         <is>
-          <t>http://tsb-bst.gc.ca/eng/divulgation-disclosure/infosource/index.asp</t>
+          <t>https://www.tsb.gc.ca/eng/divulgation-disclosure/infosource/index.html</t>
         </is>
       </c>
       <c r="BZ55" t="inlineStr">
         <is>
-          <t>http://tsb-bst.gc.ca/fra/divulgation-disclosure/infosource/index.asp</t>
+          <t>https://www.tsb.gc.ca/fra/divulgation-disclosure/infosource/index.html</t>
         </is>
       </c>
       <c r="CA55" t="inlineStr">
         <is>
-          <t>http://tsb-bst.gc.ca/fra/divulgation-disclosure/infosource/index.asp</t>
+          <t>https://www.tsb.gc.ca/fra/divulgation-disclosure/infosource/index.html</t>
         </is>
       </c>
       <c r="CB55" t="inlineStr">
@@ -21298,12 +21334,12 @@
       </c>
       <c r="CF55" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/list-institutions.html</t>
+          <t>https://www.tsb.gc.ca/eng/divulgation-disclosure/infosource/index.html</t>
         </is>
       </c>
       <c r="CG55" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/liste-organisations.html</t>
+          <t>https://www.tsb.gc.ca/fra/divulgation-disclosure/infosource/index.html</t>
         </is>
       </c>
       <c r="CH55" t="inlineStr">
@@ -21328,7 +21364,7 @@
       </c>
       <c r="CL55" t="inlineStr">
         <is>
-          <t>reachable_unverified_content</t>
+          <t>verified_info_source</t>
         </is>
       </c>
       <c r="CM55" t="n">
@@ -21336,12 +21372,12 @@
       </c>
       <c r="CN55" t="inlineStr">
         <is>
-          <t>https://tsb-bst.gc.ca/splash?destination=/homepage</t>
+          <t>https://www.tsb.gc.ca/eng/divulgation-disclosure/infosource/index.html</t>
         </is>
       </c>
       <c r="CO55" t="inlineStr">
         <is>
-          <t>reachable_unverified_content</t>
+          <t>verified_info_source</t>
         </is>
       </c>
       <c r="CP55" t="n">
@@ -21349,7 +21385,7 @@
       </c>
       <c r="CQ55" t="inlineStr">
         <is>
-          <t>https://tsb-bst.gc.ca/splash?destination=/homepage</t>
+          <t>https://www.tsb.gc.ca/fra/divulgation-disclosure/infosource/index.html</t>
         </is>
       </c>
     </row>
@@ -38445,15 +38481,51 @@
       <c r="BH105" t="inlineStr"/>
       <c r="BI105" t="inlineStr"/>
       <c r="BJ105" t="inlineStr"/>
-      <c r="BK105" t="inlineStr"/>
-      <c r="BL105" t="inlineStr"/>
-      <c r="BM105" t="inlineStr"/>
-      <c r="BN105" t="inlineStr"/>
-      <c r="BO105" t="inlineStr"/>
-      <c r="BP105" t="inlineStr"/>
-      <c r="BQ105" t="inlineStr"/>
-      <c r="BR105" t="inlineStr"/>
-      <c r="BS105" t="inlineStr"/>
+      <c r="BK105" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/auditor-general/transparency/info-source/sources-federal-government-employee-information.html</t>
+        </is>
+      </c>
+      <c r="BL105" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/verificateur-general/transparence/info-source/sources-renseignements-gouvernement-federal-fonctionnaires-federaux.html</t>
+        </is>
+      </c>
+      <c r="BM105" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/auditor-general/transparency/info-source/sources-federal-government-employee-information.html</t>
+        </is>
+      </c>
+      <c r="BN105" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/verificateur-general/transparence/info-source/sources-renseignements-gouvernement-federal-fonctionnaires-federaux.html</t>
+        </is>
+      </c>
+      <c r="BO105" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/auditor-general/transparency/info-source/sources-federal-government-employee-information.html</t>
+        </is>
+      </c>
+      <c r="BP105" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/verificateur-general/transparence/info-source/sources-renseignements-gouvernement-federal-fonctionnaires-federaux.html</t>
+        </is>
+      </c>
+      <c r="BQ105" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/auditor-general/transparency/info-source/sources-federal-government-employee-information.html</t>
+        </is>
+      </c>
+      <c r="BR105" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/verificateur-general/transparence/info-source/sources-renseignements-gouvernement-federal-fonctionnaires-federaux.html</t>
+        </is>
+      </c>
+      <c r="BS105" t="inlineStr">
+        <is>
+          <t>Current bilingual Canada.ca publication replaces legacy OAG pages that returned non-substantive content.</t>
+        </is>
+      </c>
       <c r="BT105" t="inlineStr">
         <is>
           <t>09-30</t>
@@ -38466,32 +38538,32 @@
       </c>
       <c r="BV105" t="inlineStr">
         <is>
-          <t>http://www.oag-bvg.gc.ca/internet/English/acc_fs_e_38857.html</t>
+          <t>https://www.canada.ca/en/auditor-general/transparency/info-source/sources-federal-government-employee-information.html</t>
         </is>
       </c>
       <c r="BW105" t="inlineStr">
         <is>
-          <t>http://www.oag-bvg.gc.ca/internet/Francais/acc_fs_f_38857.html</t>
+          <t>https://www.canada.ca/fr/verificateur-general/transparence/info-source/sources-renseignements-gouvernement-federal-fonctionnaires-federaux.html</t>
         </is>
       </c>
       <c r="BX105" t="inlineStr">
         <is>
-          <t>http://www.oag-bvg.gc.ca/internet/English/acc_fs_e_38857.html</t>
+          <t>https://www.canada.ca/en/auditor-general/transparency/info-source/sources-federal-government-employee-information.html</t>
         </is>
       </c>
       <c r="BY105" t="inlineStr">
         <is>
-          <t>http://www.oag-bvg.gc.ca/internet/English/acc_fs_e_38857.html</t>
+          <t>https://www.canada.ca/en/auditor-general/transparency/info-source/sources-federal-government-employee-information.html</t>
         </is>
       </c>
       <c r="BZ105" t="inlineStr">
         <is>
-          <t>http://www.oag-bvg.gc.ca/internet/Francais/acc_fs_f_38857.html</t>
+          <t>https://www.canada.ca/fr/verificateur-general/transparence/info-source/sources-renseignements-gouvernement-federal-fonctionnaires-federaux.html</t>
         </is>
       </c>
       <c r="CA105" t="inlineStr">
         <is>
-          <t>http://www.oag-bvg.gc.ca/internet/Francais/acc_fs_f_38857.html</t>
+          <t>https://www.canada.ca/fr/verificateur-general/transparence/info-source/sources-renseignements-gouvernement-federal-fonctionnaires-federaux.html</t>
         </is>
       </c>
       <c r="CB105" t="inlineStr">
@@ -38516,12 +38588,12 @@
       </c>
       <c r="CF105" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/list-institutions.html</t>
+          <t>https://www.canada.ca/en/auditor-general/transparency/info-source/sources-federal-government-employee-information.html</t>
         </is>
       </c>
       <c r="CG105" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/liste-organisations.html</t>
+          <t>https://www.canada.ca/fr/verificateur-general/transparence/info-source/sources-renseignements-gouvernement-federal-fonctionnaires-federaux.html</t>
         </is>
       </c>
       <c r="CH105" t="inlineStr">
@@ -38546,7 +38618,7 @@
       </c>
       <c r="CL105" t="inlineStr">
         <is>
-          <t>reachable_unverified_content</t>
+          <t>verified_info_source</t>
         </is>
       </c>
       <c r="CM105" t="n">
@@ -38554,12 +38626,12 @@
       </c>
       <c r="CN105" t="inlineStr">
         <is>
-          <t>https://www.oag-bvg.gc.ca/internet/English/acc_fs_e_38857.html</t>
+          <t>https://www.canada.ca/en/auditor-general/transparency/info-source/sources-federal-government-employee-information.html</t>
         </is>
       </c>
       <c r="CO105" t="inlineStr">
         <is>
-          <t>reachable_unverified_content</t>
+          <t>verified_info_source</t>
         </is>
       </c>
       <c r="CP105" t="n">
@@ -38567,7 +38639,7 @@
       </c>
       <c r="CQ105" t="inlineStr">
         <is>
-          <t>https://www.oag-bvg.gc.ca/internet/Francais/acc_fs_f_38857.html</t>
+          <t>https://www.canada.ca/fr/verificateur-general/transparence/info-source/sources-renseignements-gouvernement-federal-fonctionnaires-federaux.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh CSPS and C-NLOER Info Source data
</commit_message>
<xml_diff>
--- a/institution_registry.xlsx
+++ b/institution_registry.xlsx
@@ -13286,15 +13286,51 @@
       <c r="BH34" t="inlineStr"/>
       <c r="BI34" t="inlineStr"/>
       <c r="BJ34" t="inlineStr"/>
-      <c r="BK34" t="inlineStr"/>
-      <c r="BL34" t="inlineStr"/>
-      <c r="BM34" t="inlineStr"/>
-      <c r="BN34" t="inlineStr"/>
-      <c r="BO34" t="inlineStr"/>
-      <c r="BP34" t="inlineStr"/>
-      <c r="BQ34" t="inlineStr"/>
-      <c r="BR34" t="inlineStr"/>
-      <c r="BS34" t="inlineStr"/>
+      <c r="BK34" t="inlineStr">
+        <is>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource.pdf</t>
+        </is>
+      </c>
+      <c r="BL34" t="inlineStr">
+        <is>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource_fr.pdf</t>
+        </is>
+      </c>
+      <c r="BM34" t="inlineStr">
+        <is>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource.pdf</t>
+        </is>
+      </c>
+      <c r="BN34" t="inlineStr">
+        <is>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource_fr.pdf</t>
+        </is>
+      </c>
+      <c r="BO34" t="inlineStr">
+        <is>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource.pdf</t>
+        </is>
+      </c>
+      <c r="BP34" t="inlineStr">
+        <is>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource_fr.pdf</t>
+        </is>
+      </c>
+      <c r="BQ34" t="inlineStr">
+        <is>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource.pdf</t>
+        </is>
+      </c>
+      <c r="BR34" t="inlineStr">
+        <is>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource_fr.pdf</t>
+        </is>
+      </c>
+      <c r="BS34" t="inlineStr">
+        <is>
+          <t>Current bilingual institution PDFs replace the English-only Info Source landing page.</t>
+        </is>
+      </c>
       <c r="BT34" t="inlineStr">
         <is>
           <t>03-31</t>
@@ -13307,22 +13343,34 @@
       </c>
       <c r="BV34" t="inlineStr">
         <is>
-          <t>https://www.cnlopb.ca/information/infosource/</t>
-        </is>
-      </c>
-      <c r="BW34" t="inlineStr"/>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource.pdf</t>
+        </is>
+      </c>
+      <c r="BW34" t="inlineStr">
+        <is>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource_fr.pdf</t>
+        </is>
+      </c>
       <c r="BX34" t="inlineStr">
         <is>
-          <t>https://www.cnlopb.ca/information/infosource/</t>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource.pdf</t>
         </is>
       </c>
       <c r="BY34" t="inlineStr">
         <is>
-          <t>https://www.cnlopb.ca/information/infosource/</t>
-        </is>
-      </c>
-      <c r="BZ34" t="inlineStr"/>
-      <c r="CA34" t="inlineStr"/>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource.pdf</t>
+        </is>
+      </c>
+      <c r="BZ34" t="inlineStr">
+        <is>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource_fr.pdf</t>
+        </is>
+      </c>
+      <c r="CA34" t="inlineStr">
+        <is>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource_fr.pdf</t>
+        </is>
+      </c>
       <c r="CB34" t="inlineStr">
         <is>
           <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/access-informatio-policies-guidance/programs-holdings-online-publishing-requirements.html#toc-a</t>
@@ -13345,10 +13393,14 @@
       </c>
       <c r="CF34" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/list-institutions.html</t>
-        </is>
-      </c>
-      <c r="CG34" t="inlineStr"/>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource.pdf</t>
+        </is>
+      </c>
+      <c r="CG34" t="inlineStr">
+        <is>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource_fr.pdf</t>
+        </is>
+      </c>
       <c r="CH34" t="inlineStr">
         <is>
           <t>https://open.canada.ca/data/api/action/organization_list?all_fields=true&amp;include_extras=true</t>
@@ -13371,7 +13423,7 @@
       </c>
       <c r="CL34" t="inlineStr">
         <is>
-          <t>reachable_unverified_content</t>
+          <t>reachable_pdf</t>
         </is>
       </c>
       <c r="CM34" t="n">
@@ -13379,16 +13431,22 @@
       </c>
       <c r="CN34" t="inlineStr">
         <is>
-          <t>https://www.cnlopb.ca/information/infosource/</t>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource.pdf</t>
         </is>
       </c>
       <c r="CO34" t="inlineStr">
         <is>
-          <t>missing_url</t>
-        </is>
-      </c>
-      <c r="CP34" t="inlineStr"/>
-      <c r="CQ34" t="inlineStr"/>
+          <t>reachable_pdf</t>
+        </is>
+      </c>
+      <c r="CP34" t="n">
+        <v>200</v>
+      </c>
+      <c r="CQ34" t="inlineStr">
+        <is>
+          <t>https://www.cnlopb.ca/wp-content/uploads/InfoSource_fr.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -14375,15 +14433,51 @@
       <c r="BH37" t="inlineStr"/>
       <c r="BI37" t="inlineStr"/>
       <c r="BJ37" t="inlineStr"/>
-      <c r="BK37" t="inlineStr"/>
-      <c r="BL37" t="inlineStr"/>
-      <c r="BM37" t="inlineStr"/>
-      <c r="BN37" t="inlineStr"/>
-      <c r="BO37" t="inlineStr"/>
-      <c r="BP37" t="inlineStr"/>
-      <c r="BQ37" t="inlineStr"/>
-      <c r="BR37" t="inlineStr"/>
-      <c r="BS37" t="inlineStr"/>
+      <c r="BK37" t="inlineStr">
+        <is>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-eng.aspx</t>
+        </is>
+      </c>
+      <c r="BL37" t="inlineStr">
+        <is>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-fra.aspx</t>
+        </is>
+      </c>
+      <c r="BM37" t="inlineStr">
+        <is>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-eng.aspx</t>
+        </is>
+      </c>
+      <c r="BN37" t="inlineStr">
+        <is>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-fra.aspx</t>
+        </is>
+      </c>
+      <c r="BO37" t="inlineStr">
+        <is>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-eng.aspx</t>
+        </is>
+      </c>
+      <c r="BP37" t="inlineStr">
+        <is>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-fra.aspx</t>
+        </is>
+      </c>
+      <c r="BQ37" t="inlineStr">
+        <is>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-eng.aspx</t>
+        </is>
+      </c>
+      <c r="BR37" t="inlineStr">
+        <is>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-fra.aspx</t>
+        </is>
+      </c>
+      <c r="BS37" t="inlineStr">
+        <is>
+          <t>Current bilingual Info Source pages replace legacy program-and-holdings routes that redirect to an error page.</t>
+        </is>
+      </c>
       <c r="BT37" t="inlineStr">
         <is>
           <t>06-30</t>
@@ -14396,32 +14490,32 @@
       </c>
       <c r="BV37" t="inlineStr">
         <is>
-          <t>https://csps-efpc.gc.ca/About_Us/currentreport/programs-holdings-eng.aspx</t>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-eng.aspx</t>
         </is>
       </c>
       <c r="BW37" t="inlineStr">
         <is>
-          <t>https://csps-efpc.gc.ca/about_us/currentreport/programs-holdings-fra.aspx</t>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-fra.aspx</t>
         </is>
       </c>
       <c r="BX37" t="inlineStr">
         <is>
-          <t>https://csps-efpc.gc.ca/About_Us/currentreport/programs-holdings-eng.aspx</t>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-eng.aspx</t>
         </is>
       </c>
       <c r="BY37" t="inlineStr">
         <is>
-          <t>https://csps-efpc.gc.ca/About_Us/currentreport/programs-holdings-eng.aspx</t>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-eng.aspx</t>
         </is>
       </c>
       <c r="BZ37" t="inlineStr">
         <is>
-          <t>https://csps-efpc.gc.ca/about_us/currentreport/programs-holdings-fra.aspx</t>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-fra.aspx</t>
         </is>
       </c>
       <c r="CA37" t="inlineStr">
         <is>
-          <t>https://csps-efpc.gc.ca/about_us/currentreport/programs-holdings-fra.aspx</t>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-fra.aspx</t>
         </is>
       </c>
       <c r="CB37" t="inlineStr">
@@ -14446,12 +14540,12 @@
       </c>
       <c r="CF37" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/list-institutions.html</t>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-eng.aspx</t>
         </is>
       </c>
       <c r="CG37" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/liste-organisations.html</t>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-fra.aspx</t>
         </is>
       </c>
       <c r="CH37" t="inlineStr">
@@ -14476,7 +14570,7 @@
       </c>
       <c r="CL37" t="inlineStr">
         <is>
-          <t>reachable_unverified_content</t>
+          <t>verified_info_source</t>
         </is>
       </c>
       <c r="CM37" t="n">
@@ -14484,12 +14578,12 @@
       </c>
       <c r="CN37" t="inlineStr">
         <is>
-          <t>https://www.csps-efpc.gc.ca/error/default.aspx?aspxerrorpath=/about_us/currentreport/programs-holdings-eng.aspx</t>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-eng.aspx</t>
         </is>
       </c>
       <c r="CO37" t="inlineStr">
         <is>
-          <t>reachable_unverified_content</t>
+          <t>verified_info_source</t>
         </is>
       </c>
       <c r="CP37" t="n">
@@ -14497,7 +14591,7 @@
       </c>
       <c r="CQ37" t="inlineStr">
         <is>
-          <t>https://www.csps-efpc.gc.ca/error/default.aspx?aspxerrorpath=/about_us/currentreport/programs-holdings-fra.aspx</t>
+          <t>https://www.csps-efpc.gc.ca/about_us/currentreport/infosource-fra.aspx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh WAGE NFB and NFPC Info Source data
</commit_message>
<xml_diff>
--- a/institution_registry.xlsx
+++ b/institution_registry.xlsx
@@ -1162,17 +1162,49 @@
       <c r="BH2" t="inlineStr"/>
       <c r="BI2" t="inlineStr"/>
       <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="inlineStr"/>
-      <c r="BM2" t="inlineStr"/>
-      <c r="BN2" t="inlineStr"/>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
-      <c r="BQ2" t="inlineStr"/>
-      <c r="BR2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/women-gender-equality/transparency/annual-report-parliament-access-information-privacy/info-source-2024-2025.html</t>
+        </is>
+      </c>
+      <c r="BL2" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/femmes-egalite-genres/transparence/rapport-annuel-parlement-acces-information-protection-renseignements-personnels/info-source-2024-2025.html</t>
+        </is>
+      </c>
+      <c r="BM2" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/women-gender-equality/transparency/annual-report-parliament-access-information-privacy/info-source-2024-2025.html</t>
+        </is>
+      </c>
+      <c r="BN2" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/femmes-egalite-genres/transparence/rapport-annuel-parlement-acces-information-protection-renseignements-personnels/info-source-2024-2025.html</t>
+        </is>
+      </c>
+      <c r="BO2" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/women-gender-equality/transparency/annual-report-parliament-access-information-privacy/info-source-2024-2025.html</t>
+        </is>
+      </c>
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/femmes-egalite-genres/transparence/rapport-annuel-parlement-acces-information-protection-renseignements-personnels/info-source-2024-2025.html</t>
+        </is>
+      </c>
+      <c r="BQ2" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/women-gender-equality/transparency/annual-report-parliament-access-information-privacy/info-source-2024-2025.html</t>
+        </is>
+      </c>
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/femmes-egalite-genres/transparence/rapport-annuel-parlement-acces-information-protection-renseignements-personnels/info-source-2024-2025.html</t>
+        </is>
+      </c>
       <c r="BS2" t="inlineStr">
         <is>
-          <t>Current legal and public-facing names differ.</t>
+          <t>Current bilingual 2024-2025 Info Source replaces the 2023-2024 publication; legal and public-facing names differ.</t>
         </is>
       </c>
       <c r="BT2" t="inlineStr">
@@ -1187,32 +1219,32 @@
       </c>
       <c r="BV2" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/women-gender-equality/transparency/annual-report-parliament-access-information-privacy/info-source-2023-2024.html</t>
+          <t>https://www.canada.ca/en/women-gender-equality/transparency/annual-report-parliament-access-information-privacy/info-source-2024-2025.html</t>
         </is>
       </c>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/femmes-egalite-genres/transparence/rapport-annuel-parlement-acces-information-protection-renseignements-personnels/info-source-2023-2024.html</t>
+          <t>https://www.canada.ca/fr/femmes-egalite-genres/transparence/rapport-annuel-parlement-acces-information-protection-renseignements-personnels/info-source-2024-2025.html</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/women-gender-equality/transparency/annual-report-parliament-access-information-privacy/info-source-2023-2024.html</t>
+          <t>https://www.canada.ca/en/women-gender-equality/transparency/annual-report-parliament-access-information-privacy/info-source-2024-2025.html</t>
         </is>
       </c>
       <c r="BY2" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/women-gender-equality/transparency/annual-report-parliament-access-information-privacy/info-source-2023-2024.html</t>
+          <t>https://www.canada.ca/en/women-gender-equality/transparency/annual-report-parliament-access-information-privacy/info-source-2024-2025.html</t>
         </is>
       </c>
       <c r="BZ2" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/femmes-egalite-genres/transparence/rapport-annuel-parlement-acces-information-protection-renseignements-personnels/info-source-2023-2024.html</t>
+          <t>https://www.canada.ca/fr/femmes-egalite-genres/transparence/rapport-annuel-parlement-acces-information-protection-renseignements-personnels/info-source-2024-2025.html</t>
         </is>
       </c>
       <c r="CA2" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/femmes-egalite-genres/transparence/rapport-annuel-parlement-acces-information-protection-renseignements-personnels/info-source-2023-2024.html</t>
+          <t>https://www.canada.ca/fr/femmes-egalite-genres/transparence/rapport-annuel-parlement-acces-information-protection-renseignements-personnels/info-source-2024-2025.html</t>
         </is>
       </c>
       <c r="CB2" t="inlineStr">
@@ -1237,12 +1269,12 @@
       </c>
       <c r="CF2" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/list-institutions.html</t>
+          <t>https://www.canada.ca/en/women-gender-equality/transparency/annual-report-parliament-access-information-privacy/info-source-2024-2025.html</t>
         </is>
       </c>
       <c r="CG2" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/liste-organisations.html</t>
+          <t>https://www.canada.ca/fr/femmes-egalite-genres/transparence/rapport-annuel-parlement-acces-information-protection-renseignements-personnels/info-source-2024-2025.html</t>
         </is>
       </c>
       <c r="CH2" t="inlineStr">
@@ -1275,7 +1307,7 @@
       </c>
       <c r="CN2" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/women-gender-equality/transparency/annual-report-parliament-access-information-privacy/info-source-2023-2024.html</t>
+          <t>https://www.canada.ca/en/women-gender-equality/transparency/annual-report-parliament-access-information-privacy/info-source-2024-2025.html</t>
         </is>
       </c>
       <c r="CO2" t="inlineStr">
@@ -1288,7 +1320,7 @@
       </c>
       <c r="CQ2" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/femmes-egalite-genres/transparence/rapport-annuel-parlement-acces-information-protection-renseignements-personnels/info-source-2023-2024.html</t>
+          <t>https://www.canada.ca/fr/femmes-egalite-genres/transparence/rapport-annuel-parlement-acces-information-protection-renseignements-personnels/info-source-2024-2025.html</t>
         </is>
       </c>
     </row>
@@ -17475,15 +17507,35 @@
       <c r="BH45" t="inlineStr"/>
       <c r="BI45" t="inlineStr"/>
       <c r="BJ45" t="inlineStr"/>
-      <c r="BK45" t="inlineStr"/>
-      <c r="BL45" t="inlineStr"/>
+      <c r="BK45" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/polar-knowledge/infosource.html</t>
+        </is>
+      </c>
+      <c r="BL45" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/savoir-polaire/infosource.html</t>
+        </is>
+      </c>
       <c r="BM45" t="inlineStr"/>
       <c r="BN45" t="inlineStr"/>
       <c r="BO45" t="inlineStr"/>
       <c r="BP45" t="inlineStr"/>
-      <c r="BQ45" t="inlineStr"/>
-      <c r="BR45" t="inlineStr"/>
-      <c r="BS45" t="inlineStr"/>
+      <c r="BQ45" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/polar-knowledge/infosource.html</t>
+        </is>
+      </c>
+      <c r="BR45" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/savoir-polaire/infosource.html</t>
+        </is>
+      </c>
+      <c r="BS45" t="inlineStr">
+        <is>
+          <t>Owner-supplied bilingual Info Source URLs; neither page supplies institution-specific PIB or class details.</t>
+        </is>
+      </c>
       <c r="BT45" t="inlineStr">
         <is>
           <t>03-31</t>
@@ -17496,34 +17548,18 @@
       </c>
       <c r="BV45" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/polar-knowledge/proactivedisclosure.html</t>
+          <t>https://www.canada.ca/en/polar-knowledge/infosource.html</t>
         </is>
       </c>
       <c r="BW45" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/savoir-polaire/divulgationproactive.html</t>
-        </is>
-      </c>
-      <c r="BX45" t="inlineStr">
-        <is>
-          <t>https://www.canada.ca/en/polar-knowledge/proactivedisclosure.html</t>
-        </is>
-      </c>
-      <c r="BY45" t="inlineStr">
-        <is>
-          <t>https://www.canada.ca/en/polar-knowledge/proactivedisclosure.html</t>
-        </is>
-      </c>
-      <c r="BZ45" t="inlineStr">
-        <is>
-          <t>https://www.canada.ca/fr/savoir-polaire/divulgationproactive.html</t>
-        </is>
-      </c>
-      <c r="CA45" t="inlineStr">
-        <is>
-          <t>https://www.canada.ca/fr/savoir-polaire/divulgationproactive.html</t>
-        </is>
-      </c>
+          <t>https://www.canada.ca/fr/savoir-polaire/infosource.html</t>
+        </is>
+      </c>
+      <c r="BX45" t="inlineStr"/>
+      <c r="BY45" t="inlineStr"/>
+      <c r="BZ45" t="inlineStr"/>
+      <c r="CA45" t="inlineStr"/>
       <c r="CB45" t="inlineStr">
         <is>
           <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/access-informatio-policies-guidance/programs-holdings-online-publishing-requirements.html#toc-a</t>
@@ -17546,12 +17582,12 @@
       </c>
       <c r="CF45" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/list-institutions.html</t>
+          <t>https://www.canada.ca/en/polar-knowledge/infosource.html</t>
         </is>
       </c>
       <c r="CG45" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/liste-organisations.html</t>
+          <t>https://www.canada.ca/fr/savoir-polaire/infosource.html</t>
         </is>
       </c>
       <c r="CH45" t="inlineStr">
@@ -17584,20 +17620,20 @@
       </c>
       <c r="CN45" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/polar-knowledge/proactivedisclosure.html</t>
+          <t>https://www.canada.ca/en/polar-knowledge/infosource.html</t>
         </is>
       </c>
       <c r="CO45" t="inlineStr">
         <is>
-          <t>reachable_unverified_content</t>
+          <t>http_error</t>
         </is>
       </c>
       <c r="CP45" t="n">
-        <v>200</v>
+        <v>404</v>
       </c>
       <c r="CQ45" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/savoir-polaire/divulgationproactive.html</t>
+          <t>https://www.canada.ca/fr/savoir-polaire/infosource.html</t>
         </is>
       </c>
     </row>
@@ -34449,15 +34485,51 @@
       <c r="BH93" t="inlineStr"/>
       <c r="BI93" t="inlineStr"/>
       <c r="BJ93" t="inlineStr"/>
-      <c r="BK93" t="inlineStr"/>
-      <c r="BL93" t="inlineStr"/>
-      <c r="BM93" t="inlineStr"/>
-      <c r="BN93" t="inlineStr"/>
-      <c r="BO93" t="inlineStr"/>
-      <c r="BP93" t="inlineStr"/>
-      <c r="BQ93" t="inlineStr"/>
-      <c r="BR93" t="inlineStr"/>
-      <c r="BS93" t="inlineStr"/>
+      <c r="BK93" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/farm-products-council/corporate/about/transparency/info-source-fpcc.html</t>
+        </is>
+      </c>
+      <c r="BL93" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/conseil-produits-agricoles/entreprise/propos/transparence/info-source-cpac.html</t>
+        </is>
+      </c>
+      <c r="BM93" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/farm-products-council/corporate/about/transparency/info-source-fpcc.html</t>
+        </is>
+      </c>
+      <c r="BN93" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/conseil-produits-agricoles/entreprise/propos/transparence/info-source-cpac.html</t>
+        </is>
+      </c>
+      <c r="BO93" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/farm-products-council/corporate/about/transparency/info-source-fpcc.html</t>
+        </is>
+      </c>
+      <c r="BP93" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/conseil-produits-agricoles/entreprise/propos/transparence/info-source-cpac.html</t>
+        </is>
+      </c>
+      <c r="BQ93" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/farm-products-council/corporate/about/transparency/info-source-fpcc.html</t>
+        </is>
+      </c>
+      <c r="BR93" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/conseil-produits-agricoles/entreprise/propos/transparence/info-source-cpac.html</t>
+        </is>
+      </c>
+      <c r="BS93" t="inlineStr">
+        <is>
+          <t>Current bilingual Info Source overview pages replace obsolete proactive-disclosure URLs; numbered holdings are not present on these pages.</t>
+        </is>
+      </c>
       <c r="BT93" t="inlineStr">
         <is>
           <t>09-30</t>
@@ -34470,32 +34542,32 @@
       </c>
       <c r="BV93" t="inlineStr">
         <is>
-          <t>http://fpcc-cpac.gc.ca/index.php/en-GB/proactive-disclosures</t>
+          <t>https://www.canada.ca/en/farm-products-council/corporate/about/transparency/info-source-fpcc.html</t>
         </is>
       </c>
       <c r="BW93" t="inlineStr">
         <is>
-          <t>http://fpcc-cpac.gc.ca/index.php/fr-FR/divulgations-proactive</t>
+          <t>https://www.canada.ca/fr/conseil-produits-agricoles/entreprise/propos/transparence/info-source-cpac.html</t>
         </is>
       </c>
       <c r="BX93" t="inlineStr">
         <is>
-          <t>http://fpcc-cpac.gc.ca/index.php/en-GB/proactive-disclosures</t>
+          <t>https://www.canada.ca/en/farm-products-council/corporate/about/transparency/info-source-fpcc.html</t>
         </is>
       </c>
       <c r="BY93" t="inlineStr">
         <is>
-          <t>http://fpcc-cpac.gc.ca/index.php/en-GB/proactive-disclosures</t>
+          <t>https://www.canada.ca/en/farm-products-council/corporate/about/transparency/info-source-fpcc.html</t>
         </is>
       </c>
       <c r="BZ93" t="inlineStr">
         <is>
-          <t>http://fpcc-cpac.gc.ca/index.php/fr-FR/divulgations-proactive</t>
+          <t>https://www.canada.ca/fr/conseil-produits-agricoles/entreprise/propos/transparence/info-source-cpac.html</t>
         </is>
       </c>
       <c r="CA93" t="inlineStr">
         <is>
-          <t>http://fpcc-cpac.gc.ca/index.php/fr-FR/divulgations-proactive</t>
+          <t>https://www.canada.ca/fr/conseil-produits-agricoles/entreprise/propos/transparence/info-source-cpac.html</t>
         </is>
       </c>
       <c r="CB93" t="inlineStr">
@@ -34520,12 +34592,12 @@
       </c>
       <c r="CF93" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/list-institutions.html</t>
+          <t>https://www.canada.ca/en/farm-products-council/corporate/about/transparency/info-source-fpcc.html</t>
         </is>
       </c>
       <c r="CG93" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/liste-organisations.html</t>
+          <t>https://www.canada.ca/fr/conseil-produits-agricoles/entreprise/propos/transparence/info-source-cpac.html</t>
         </is>
       </c>
       <c r="CH93" t="inlineStr">
@@ -34550,18 +34622,30 @@
       </c>
       <c r="CL93" t="inlineStr">
         <is>
-          <t>request_error</t>
-        </is>
-      </c>
-      <c r="CM93" t="inlineStr"/>
-      <c r="CN93" t="inlineStr"/>
+          <t>verified_info_source</t>
+        </is>
+      </c>
+      <c r="CM93" t="n">
+        <v>200</v>
+      </c>
+      <c r="CN93" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/farm-products-council/corporate/about/transparency/info-source-fpcc.html</t>
+        </is>
+      </c>
       <c r="CO93" t="inlineStr">
         <is>
-          <t>request_error</t>
-        </is>
-      </c>
-      <c r="CP93" t="inlineStr"/>
-      <c r="CQ93" t="inlineStr"/>
+          <t>verified_info_source</t>
+        </is>
+      </c>
+      <c r="CP93" t="n">
+        <v>200</v>
+      </c>
+      <c r="CQ93" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/conseil-produits-agricoles/entreprise/propos/transparence/info-source-cpac.html</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -34824,17 +34908,49 @@
       <c r="BH94" t="inlineStr"/>
       <c r="BI94" t="inlineStr"/>
       <c r="BJ94" t="inlineStr"/>
-      <c r="BK94" t="inlineStr"/>
-      <c r="BL94" t="inlineStr"/>
-      <c r="BM94" t="inlineStr"/>
-      <c r="BN94" t="inlineStr"/>
-      <c r="BO94" t="inlineStr"/>
-      <c r="BP94" t="inlineStr"/>
-      <c r="BQ94" t="inlineStr"/>
-      <c r="BR94" t="inlineStr"/>
+      <c r="BK94" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/national-film-board/corporate/publications/general-publications/info-source.html</t>
+        </is>
+      </c>
+      <c r="BL94" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/office-national-film/organisation/publications/publications-generales/info-source.html</t>
+        </is>
+      </c>
+      <c r="BM94" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/national-film-board/corporate/publications/general-publications/info-source.html</t>
+        </is>
+      </c>
+      <c r="BN94" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/office-national-film/organisation/publications/publications-generales/info-source.html</t>
+        </is>
+      </c>
+      <c r="BO94" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/national-film-board/corporate/publications/general-publications/info-source.html</t>
+        </is>
+      </c>
+      <c r="BP94" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/office-national-film/organisation/publications/publications-generales/info-source.html</t>
+        </is>
+      </c>
+      <c r="BQ94" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/national-film-board/corporate/publications/general-publications/info-source.html</t>
+        </is>
+      </c>
+      <c r="BR94" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/office-national-film/organisation/publications/publications-generales/info-source.html</t>
+        </is>
+      </c>
       <c r="BS94" t="inlineStr">
         <is>
-          <t>Public-facing name includes Canada.</t>
+          <t>Current bilingual Info Source pages replace obsolete institution-domain URLs; public-facing name includes Canada.</t>
         </is>
       </c>
       <c r="BT94" t="inlineStr">
@@ -34849,32 +34965,32 @@
       </c>
       <c r="BV94" t="inlineStr">
         <is>
-          <t>http://onf-nfb.gc.ca/en/about-the-nfb/publications/info-source/</t>
+          <t>https://www.canada.ca/en/national-film-board/corporate/publications/general-publications/info-source.html</t>
         </is>
       </c>
       <c r="BW94" t="inlineStr">
         <is>
-          <t>http://onf-nfb.gc.ca/fr/a-propos-de-lonf/publications/info-source/</t>
+          <t>https://www.canada.ca/fr/office-national-film/organisation/publications/publications-generales/info-source.html</t>
         </is>
       </c>
       <c r="BX94" t="inlineStr">
         <is>
-          <t>http://onf-nfb.gc.ca/en/about-the-nfb/publications/info-source/</t>
+          <t>https://www.canada.ca/en/national-film-board/corporate/publications/general-publications/info-source.html</t>
         </is>
       </c>
       <c r="BY94" t="inlineStr">
         <is>
-          <t>http://onf-nfb.gc.ca/en/about-the-nfb/publications/info-source/</t>
+          <t>https://www.canada.ca/en/national-film-board/corporate/publications/general-publications/info-source.html</t>
         </is>
       </c>
       <c r="BZ94" t="inlineStr">
         <is>
-          <t>http://onf-nfb.gc.ca/fr/a-propos-de-lonf/publications/info-source/</t>
+          <t>https://www.canada.ca/fr/office-national-film/organisation/publications/publications-generales/info-source.html</t>
         </is>
       </c>
       <c r="CA94" t="inlineStr">
         <is>
-          <t>http://onf-nfb.gc.ca/fr/a-propos-de-lonf/publications/info-source/</t>
+          <t>https://www.canada.ca/fr/office-national-film/organisation/publications/publications-generales/info-source.html</t>
         </is>
       </c>
       <c r="CB94" t="inlineStr">
@@ -34899,12 +35015,12 @@
       </c>
       <c r="CF94" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/list-institutions.html</t>
+          <t>https://www.canada.ca/en/national-film-board/corporate/publications/general-publications/info-source.html</t>
         </is>
       </c>
       <c r="CG94" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/liste-organisations.html</t>
+          <t>https://www.canada.ca/fr/office-national-film/organisation/publications/publications-generales/info-source.html</t>
         </is>
       </c>
       <c r="CH94" t="inlineStr">
@@ -34929,18 +35045,30 @@
       </c>
       <c r="CL94" t="inlineStr">
         <is>
-          <t>request_error</t>
-        </is>
-      </c>
-      <c r="CM94" t="inlineStr"/>
-      <c r="CN94" t="inlineStr"/>
+          <t>verified_info_source</t>
+        </is>
+      </c>
+      <c r="CM94" t="n">
+        <v>200</v>
+      </c>
+      <c r="CN94" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/national-film-board/corporate/publications/general-publications/info-source.html</t>
+        </is>
+      </c>
       <c r="CO94" t="inlineStr">
         <is>
-          <t>request_error</t>
-        </is>
-      </c>
-      <c r="CP94" t="inlineStr"/>
-      <c r="CQ94" t="inlineStr"/>
+          <t>verified_info_source</t>
+        </is>
+      </c>
+      <c r="CP94" t="n">
+        <v>200</v>
+      </c>
+      <c r="CQ94" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/office-national-film/organisation/publications/publications-generales/info-source.html</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">

</xml_diff>

<commit_message>
Refresh AAFC, Housing, and PSPC bilingual Info Source data
</commit_message>
<xml_diff>
--- a/institution_registry.xlsx
+++ b/institution_registry.xlsx
@@ -1593,12 +1593,36 @@
       <c r="BH3" t="inlineStr"/>
       <c r="BI3" t="inlineStr"/>
       <c r="BJ3" t="inlineStr"/>
-      <c r="BK3" t="inlineStr"/>
-      <c r="BL3" t="inlineStr"/>
-      <c r="BM3" t="inlineStr"/>
-      <c r="BN3" t="inlineStr"/>
-      <c r="BO3" t="inlineStr"/>
-      <c r="BP3" t="inlineStr"/>
+      <c r="BK3" t="inlineStr">
+        <is>
+          <t>https://agriculture.canada.ca/en/department/transparency/info-source-employee-information</t>
+        </is>
+      </c>
+      <c r="BL3" t="inlineStr">
+        <is>
+          <t>https://agriculture.canada.ca/fr/ministere/transparence/info-source-renseignements-pour-fonctionnaires</t>
+        </is>
+      </c>
+      <c r="BM3" t="inlineStr">
+        <is>
+          <t>https://agriculture.canada.ca/en/department/transparency/info-source-employee-information</t>
+        </is>
+      </c>
+      <c r="BN3" t="inlineStr">
+        <is>
+          <t>https://agriculture.canada.ca/fr/ministere/transparence/info-source-renseignements-pour-fonctionnaires</t>
+        </is>
+      </c>
+      <c r="BO3" t="inlineStr">
+        <is>
+          <t>https://agriculture.canada.ca/en/department/transparency/info-source-employee-information</t>
+        </is>
+      </c>
+      <c r="BP3" t="inlineStr">
+        <is>
+          <t>https://agriculture.canada.ca/fr/ministere/transparence/info-source-renseignements-pour-fonctionnaires</t>
+        </is>
+      </c>
       <c r="BQ3" t="inlineStr"/>
       <c r="BR3" t="inlineStr"/>
       <c r="BS3" t="inlineStr"/>
@@ -1614,22 +1638,22 @@
       </c>
       <c r="BV3" t="inlineStr">
         <is>
-          <t>http://agriculture.canada.ca/eng/about-us/offices-and-locations/access-to-information-and-privacy-services/info-source-2016/?id=1347308413430</t>
+          <t>https://agriculture.canada.ca/en/department/transparency/info-source-employee-information</t>
         </is>
       </c>
       <c r="BW3" t="inlineStr">
         <is>
-          <t>http://agriculture.canada.ca/fra/a-propos-de-nous/bureaux-et-emplacements/services-dacces-a-linformation-et-de-protection-des-renseignements-personnels/sources-de-renseignements-du-gouvernement-federal-et-sur-les-fonctionnaires-federaux-2016/?id=1347308413430</t>
+          <t>https://agriculture.canada.ca/fr/ministere/transparence/info-source-renseignements-pour-fonctionnaires</t>
         </is>
       </c>
       <c r="BX3" t="inlineStr">
         <is>
-          <t>http://agriculture.canada.ca/eng/about-us/offices-and-locations/access-to-information-and-privacy-services/info-source-2016/?id=1347308413430</t>
+          <t>https://agriculture.canada.ca/en/department/transparency/info-source-employee-information</t>
         </is>
       </c>
       <c r="BY3" t="inlineStr">
         <is>
-          <t>http://agriculture.canada.ca/eng/about-us/offices-and-locations/access-to-information-and-privacy-services/info-source-2016/?id=1347308413430</t>
+          <t>https://agriculture.canada.ca/en/department/transparency/info-source-employee-information</t>
         </is>
       </c>
       <c r="BZ3" t="inlineStr">
@@ -1664,12 +1688,12 @@
       </c>
       <c r="CF3" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/list-institutions.html</t>
+          <t>https://agriculture.canada.ca/en/department/transparency/info-source-employee-information</t>
         </is>
       </c>
       <c r="CG3" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/liste-organisations.html</t>
+          <t>https://agriculture.canada.ca/fr/ministere/transparence/info-source-renseignements-pour-fonctionnaires</t>
         </is>
       </c>
       <c r="CH3" t="inlineStr">
@@ -1694,7 +1718,7 @@
       </c>
       <c r="CL3" t="inlineStr">
         <is>
-          <t>request_rejected</t>
+          <t>verified_info_source</t>
         </is>
       </c>
       <c r="CM3" t="n">
@@ -5547,12 +5571,36 @@
       <c r="BH13" t="inlineStr"/>
       <c r="BI13" t="inlineStr"/>
       <c r="BJ13" t="inlineStr"/>
-      <c r="BK13" t="inlineStr"/>
-      <c r="BL13" t="inlineStr"/>
-      <c r="BM13" t="inlineStr"/>
-      <c r="BN13" t="inlineStr"/>
-      <c r="BO13" t="inlineStr"/>
-      <c r="BP13" t="inlineStr"/>
+      <c r="BK13" t="inlineStr">
+        <is>
+          <t>https://housing-infrastructure.canada.ca/infosource/infosource-eng.html</t>
+        </is>
+      </c>
+      <c r="BL13" t="inlineStr">
+        <is>
+          <t>https://housing-infrastructure.canada.ca/infosource/infosource-fra.html</t>
+        </is>
+      </c>
+      <c r="BM13" t="inlineStr">
+        <is>
+          <t>https://housing-infrastructure.canada.ca/infosource/infosource-eng.html</t>
+        </is>
+      </c>
+      <c r="BN13" t="inlineStr">
+        <is>
+          <t>https://housing-infrastructure.canada.ca/infosource/infosource-fra.html</t>
+        </is>
+      </c>
+      <c r="BO13" t="inlineStr">
+        <is>
+          <t>https://housing-infrastructure.canada.ca/infosource/infosource-eng.html</t>
+        </is>
+      </c>
+      <c r="BP13" t="inlineStr">
+        <is>
+          <t>https://housing-infrastructure.canada.ca/infosource/infosource-fra.html</t>
+        </is>
+      </c>
       <c r="BQ13" t="inlineStr"/>
       <c r="BR13" t="inlineStr"/>
       <c r="BS13" t="inlineStr">
@@ -5572,32 +5620,32 @@
       </c>
       <c r="BV13" t="inlineStr">
         <is>
-          <t>https://www.infrastructure.gc.ca/infosource/infosource-eng.html</t>
+          <t>https://housing-infrastructure.canada.ca/infosource/infosource-eng.html</t>
         </is>
       </c>
       <c r="BW13" t="inlineStr">
         <is>
-          <t>https://www.infrastructure.gc.ca/infosource/infosource-fra.html</t>
+          <t>https://housing-infrastructure.canada.ca/infosource/infosource-fra.html</t>
         </is>
       </c>
       <c r="BX13" t="inlineStr">
         <is>
-          <t>https://www.infrastructure.gc.ca/infosource/infosource-eng.html</t>
+          <t>https://housing-infrastructure.canada.ca/infosource/infosource-eng.html</t>
         </is>
       </c>
       <c r="BY13" t="inlineStr">
         <is>
-          <t>https://www.infrastructure.gc.ca/infosource/infosource-eng.html</t>
+          <t>https://housing-infrastructure.canada.ca/infosource/infosource-eng.html</t>
         </is>
       </c>
       <c r="BZ13" t="inlineStr">
         <is>
-          <t>https://www.infrastructure.gc.ca/infosource/infosource-fra.html</t>
+          <t>https://housing-infrastructure.canada.ca/infosource/infosource-fra.html</t>
         </is>
       </c>
       <c r="CA13" t="inlineStr">
         <is>
-          <t>https://www.infrastructure.gc.ca/infosource/infosource-fra.html</t>
+          <t>https://housing-infrastructure.canada.ca/infosource/infosource-fra.html</t>
         </is>
       </c>
       <c r="CB13" t="inlineStr">
@@ -5622,12 +5670,12 @@
       </c>
       <c r="CF13" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/list-institutions.html</t>
+          <t>https://housing-infrastructure.canada.ca/infosource/infosource-eng.html</t>
         </is>
       </c>
       <c r="CG13" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/liste-organisations.html</t>
+          <t>https://housing-infrastructure.canada.ca/infosource/infosource-fra.html</t>
         </is>
       </c>
       <c r="CH13" t="inlineStr">
@@ -8304,12 +8352,36 @@
       <c r="BH20" t="inlineStr"/>
       <c r="BI20" t="inlineStr"/>
       <c r="BJ20" t="inlineStr"/>
-      <c r="BK20" t="inlineStr"/>
-      <c r="BL20" t="inlineStr"/>
-      <c r="BM20" t="inlineStr"/>
-      <c r="BN20" t="inlineStr"/>
-      <c r="BO20" t="inlineStr"/>
-      <c r="BP20" t="inlineStr"/>
+      <c r="BK20" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/public-services-procurement/corporate/transparency/access-information-privacy/understanding-your-right-obtain-information/info-source-federal-government-employee-information/about.html</t>
+        </is>
+      </c>
+      <c r="BL20" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/services-publics-approvisionnement/organisation/transparence/acces-information-protection-renseignements-personnels/comprendre-votre-droit-obtenir-renseignements/info-source-renseignements-gouvernement-federal-fonctionnaires-federaux/apropos.html</t>
+        </is>
+      </c>
+      <c r="BM20" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/public-services-procurement/corporate/transparency/access-information-privacy/understanding-your-right-obtain-information/info-source-federal-government-employee-information/institutional-program-activities.html</t>
+        </is>
+      </c>
+      <c r="BN20" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/services-publics-approvisionnement/organisation/transparence/acces-information-protection-renseignements-personnels/comprendre-votre-droit-obtenir-renseignements/info-source-renseignements-gouvernement-federal-fonctionnaires-federaux/programmes-activites-institutionnels.html</t>
+        </is>
+      </c>
+      <c r="BO20" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/public-services-procurement/corporate/transparency/access-information-privacy/understanding-your-right-obtain-information/info-source-federal-government-employee-information/institutional-program-activities.html</t>
+        </is>
+      </c>
+      <c r="BP20" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/services-publics-approvisionnement/organisation/transparence/acces-information-protection-renseignements-personnels/comprendre-votre-droit-obtenir-renseignements/info-source-renseignements-gouvernement-federal-fonctionnaires-federaux/programmes-activites-institutionnels.html</t>
+        </is>
+      </c>
       <c r="BQ20" t="inlineStr"/>
       <c r="BR20" t="inlineStr"/>
       <c r="BS20" t="inlineStr"/>
@@ -8325,32 +8397,32 @@
       </c>
       <c r="BV20" t="inlineStr">
         <is>
-          <t>http://www.tpsgc-pwgsc.gc.ca/aiprp-atip/infosource-eng.html</t>
+          <t>https://www.canada.ca/en/public-services-procurement/corporate/transparency/access-information-privacy/understanding-your-right-obtain-information/info-source-federal-government-employee-information/about.html</t>
         </is>
       </c>
       <c r="BW20" t="inlineStr">
         <is>
-          <t>http://www.tpsgc-pwgsc.gc.ca/aiprp-atip/infosource-fra.html</t>
+          <t>https://www.canada.ca/fr/services-publics-approvisionnement/organisation/transparence/acces-information-protection-renseignements-personnels/comprendre-votre-droit-obtenir-renseignements/info-source-renseignements-gouvernement-federal-fonctionnaires-federaux/apropos.html</t>
         </is>
       </c>
       <c r="BX20" t="inlineStr">
         <is>
-          <t>http://www.tpsgc-pwgsc.gc.ca/aiprp-atip/infosource-eng.html</t>
+          <t>https://www.canada.ca/en/public-services-procurement/corporate/transparency/access-information-privacy/understanding-your-right-obtain-information/info-source-federal-government-employee-information/institutional-program-activities.html</t>
         </is>
       </c>
       <c r="BY20" t="inlineStr">
         <is>
-          <t>http://www.tpsgc-pwgsc.gc.ca/aiprp-atip/infosource-eng.html</t>
+          <t>https://www.canada.ca/en/public-services-procurement/corporate/transparency/access-information-privacy/understanding-your-right-obtain-information/info-source-federal-government-employee-information/institutional-program-activities.html</t>
         </is>
       </c>
       <c r="BZ20" t="inlineStr">
         <is>
-          <t>http://www.tpsgc-pwgsc.gc.ca/aiprp-atip/infosource-fra.html</t>
+          <t>https://www.canada.ca/fr/services-publics-approvisionnement/organisation/transparence/acces-information-protection-renseignements-personnels/comprendre-votre-droit-obtenir-renseignements/info-source-renseignements-gouvernement-federal-fonctionnaires-federaux/programmes-activites-institutionnels.html</t>
         </is>
       </c>
       <c r="CA20" t="inlineStr">
         <is>
-          <t>http://www.tpsgc-pwgsc.gc.ca/aiprp-atip/infosource-fra.html</t>
+          <t>https://www.canada.ca/fr/services-publics-approvisionnement/organisation/transparence/acces-information-protection-renseignements-personnels/comprendre-votre-droit-obtenir-renseignements/info-source-renseignements-gouvernement-federal-fonctionnaires-federaux/programmes-activites-institutionnels.html</t>
         </is>
       </c>
       <c r="CB20" t="inlineStr">
@@ -8375,12 +8447,12 @@
       </c>
       <c r="CF20" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/en/treasury-board-secretariat/services/access-information-privacy/access-information/info-source/list-institutions.html</t>
+          <t>https://www.canada.ca/en/public-services-procurement/corporate/transparency/access-information-privacy/understanding-your-right-obtain-information/info-source-federal-government-employee-information/about.html</t>
         </is>
       </c>
       <c r="CG20" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/secretariat-conseil-tresor/services/acces-information-protection-reseignements-personnels/acces-information/info-source/liste-organisations.html</t>
+          <t>https://www.canada.ca/fr/services-publics-approvisionnement/organisation/transparence/acces-information-protection-renseignements-personnels/comprendre-votre-droit-obtenir-renseignements/info-source-renseignements-gouvernement-federal-fonctionnaires-federaux/apropos.html</t>
         </is>
       </c>
       <c r="CH20" t="inlineStr">
@@ -8405,18 +8477,30 @@
       </c>
       <c r="CL20" t="inlineStr">
         <is>
-          <t>request_error</t>
-        </is>
-      </c>
-      <c r="CM20" t="inlineStr"/>
-      <c r="CN20" t="inlineStr"/>
+          <t>verified_info_source</t>
+        </is>
+      </c>
+      <c r="CM20" t="n">
+        <v>200</v>
+      </c>
+      <c r="CN20" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/en/public-services-procurement/corporate/transparency/access-information-privacy/understanding-your-right-obtain-information/info-source-federal-government-employee-information/about.html</t>
+        </is>
+      </c>
       <c r="CO20" t="inlineStr">
         <is>
-          <t>request_error</t>
-        </is>
-      </c>
-      <c r="CP20" t="inlineStr"/>
-      <c r="CQ20" t="inlineStr"/>
+          <t>verified_info_source</t>
+        </is>
+      </c>
+      <c r="CP20" t="n">
+        <v>200</v>
+      </c>
+      <c r="CQ20" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/services-publics-approvisionnement/organisation/transparence/acces-information-protection-renseignements-personnels/comprendre-votre-droit-obtenir-renseignements/info-source-renseignements-gouvernement-federal-fonctionnaires-federaux/apropos.html</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">

</xml_diff>